<commit_message>
desenho e orçamento atualizaçoes ae isep
</commit_message>
<xml_diff>
--- a/DRIVE/3. Operações/3.1 Projetos/26002 - SS AEISEP (Porto)/Peças escritas/Orçamento_v2 POR-2026-0002-SSYS.xlsx
+++ b/DRIVE/3. Operações/3.1 Projetos/26002 - SS AEISEP (Porto)/Peças escritas/Orçamento_v2 POR-2026-0002-SSYS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\castr\MINDSET\DRIVE\3. Operações\3.1 Projetos\26002 - SS AEISEP (Porto)\Peças escritas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A27E01D1-6363-4F0C-B65D-1F47FCEF1BB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32E21C5D-AAF0-445E-9CBF-3377D13161BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
   <si>
     <t>DESIGNAÇÃO / DESCRIÇÃO</t>
   </si>
@@ -126,12 +126,6 @@
     <t>2º</t>
   </si>
   <si>
-    <t xml:space="preserve">Behringer Xenyx </t>
-  </si>
-  <si>
-    <t>X1832USB</t>
-  </si>
-  <si>
     <t>NOTAS: Preços por unidade apresentados não incluem IVA.Orçamento sujeito a revisões.</t>
   </si>
   <si>
@@ -190,6 +184,15 @@
   </si>
   <si>
     <t>TOTAL</t>
+  </si>
+  <si>
+    <t>Behringer Xenyx X2442 USB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aconselhada pelo projetista, mais saidas e maior compatibilidade </t>
+  </si>
+  <si>
+    <t>xx/05/2026</t>
   </si>
 </sst>
 </file>
@@ -652,9 +655,6 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="16" fontId="13" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
@@ -750,6 +750,9 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="168" fontId="25" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="16" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -1099,7 +1102,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="438" row="1">
+  <wetp:taskpane dockstate="right" visibility="0" width="438" row="2">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -1139,15 +1142,15 @@
   <sheetData>
     <row r="1" spans="1:9" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="1:9" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="32"/>
-      <c r="B2" s="33"/>
-      <c r="C2" s="33"/>
+      <c r="A2" s="31"/>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
       <c r="D2" s="75" t="s">
         <v>24</v>
       </c>
       <c r="E2" s="75"/>
       <c r="F2" s="75"/>
-      <c r="G2" s="34"/>
+      <c r="G2" s="33"/>
     </row>
     <row r="3" spans="1:9" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
@@ -1165,7 +1168,7 @@
       <c r="E4" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="57" t="s">
+      <c r="F4" s="56" t="s">
         <v>3</v>
       </c>
       <c r="G4" s="2"/>
@@ -1175,14 +1178,14 @@
       <c r="B5" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="17">
-        <v>46159</v>
+      <c r="C5" s="17" t="s">
+        <v>50</v>
       </c>
       <c r="D5" s="18"/>
       <c r="E5" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="56" t="s">
+      <c r="F5" s="55" t="s">
         <v>21</v>
       </c>
       <c r="G5" s="2"/>
@@ -1197,31 +1200,31 @@
       </c>
       <c r="D6" s="18"/>
       <c r="E6" s="19" t="s">
-        <v>48</v>
-      </c>
-      <c r="F6" s="55">
+        <v>46</v>
+      </c>
+      <c r="F6" s="54">
         <v>10</v>
       </c>
       <c r="G6" s="2"/>
     </row>
     <row r="7" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="22"/>
+      <c r="A7" s="21"/>
       <c r="B7" s="16" t="s">
         <v>11</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D7" s="18"/>
       <c r="E7" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="58" t="s">
+      <c r="F7" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="G7" s="23"/>
+      <c r="G7" s="22"/>
       <c r="H7" s="19"/>
-      <c r="I7" s="21"/>
+      <c r="I7" s="74"/>
     </row>
     <row r="8" spans="1:9" ht="3.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3"/>
@@ -1233,30 +1236,30 @@
       <c r="G8" s="5"/>
     </row>
     <row r="9" spans="1:9" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="24"/>
-      <c r="B9" s="25"/>
-      <c r="C9" s="25"/>
-      <c r="D9" s="25"/>
-      <c r="E9" s="25"/>
-      <c r="F9" s="25"/>
-      <c r="G9" s="26"/>
+      <c r="A9" s="23"/>
+      <c r="B9" s="24"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="24"/>
+      <c r="E9" s="24"/>
+      <c r="F9" s="24"/>
+      <c r="G9" s="25"/>
     </row>
     <row r="10" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
-      <c r="B10" s="35" t="s">
+      <c r="B10" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="36" t="s">
+      <c r="C10" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="D10" s="37" t="s">
+      <c r="D10" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="E10" s="38" t="s">
+      <c r="E10" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="F10" s="38" t="s">
-        <v>46</v>
+      <c r="F10" s="37" t="s">
+        <v>44</v>
       </c>
       <c r="G10" s="2"/>
     </row>
@@ -1265,19 +1268,19 @@
       <c r="B11" s="80">
         <v>1</v>
       </c>
-      <c r="C11" s="49"/>
-      <c r="D11" s="49"/>
-      <c r="E11" s="49"/>
-      <c r="F11" s="49"/>
+      <c r="C11" s="48"/>
+      <c r="D11" s="48"/>
+      <c r="E11" s="48"/>
+      <c r="F11" s="48"/>
       <c r="G11" s="10"/>
     </row>
     <row r="12" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="80"/>
-      <c r="C12" s="50" t="s">
-        <v>28</v>
-      </c>
-      <c r="D12" s="51"/>
+      <c r="C12" s="49" t="s">
+        <v>48</v>
+      </c>
+      <c r="D12" s="50"/>
       <c r="E12" s="85" t="s">
         <v>23</v>
       </c>
@@ -1287,12 +1290,12 @@
     <row r="13" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="81"/>
-      <c r="C13" s="54" t="s">
-        <v>29</v>
-      </c>
-      <c r="D13" s="52"/>
-      <c r="E13" s="52"/>
-      <c r="F13" s="52"/>
+      <c r="C13" s="53" t="s">
+        <v>49</v>
+      </c>
+      <c r="D13" s="51"/>
+      <c r="E13" s="51"/>
+      <c r="F13" s="51"/>
       <c r="G13" s="2"/>
     </row>
     <row r="14" spans="1:9" ht="6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1329,12 +1332,12 @@
     <row r="16" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="84"/>
-      <c r="C16" s="31" t="s">
+      <c r="C16" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="D16" s="27"/>
-      <c r="E16" s="27"/>
-      <c r="F16" s="27"/>
+      <c r="D16" s="26"/>
+      <c r="E16" s="26"/>
+      <c r="F16" s="26"/>
       <c r="G16" s="2"/>
     </row>
     <row r="17" spans="1:10" ht="6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1371,12 +1374,12 @@
     <row r="19" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="84"/>
-      <c r="C19" s="31" t="s">
+      <c r="C19" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="D19" s="27"/>
-      <c r="E19" s="48"/>
-      <c r="F19" s="27"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="47"/>
+      <c r="F19" s="26"/>
       <c r="G19" s="2"/>
     </row>
     <row r="20" spans="1:10" ht="6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1412,12 +1415,12 @@
     <row r="22" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="84"/>
-      <c r="C22" s="31" t="s">
+      <c r="C22" s="30" t="s">
         <v>20</v>
       </c>
-      <c r="D22" s="27"/>
-      <c r="E22" s="27"/>
-      <c r="F22" s="27"/>
+      <c r="D22" s="26"/>
+      <c r="E22" s="26"/>
+      <c r="F22" s="26"/>
       <c r="G22" s="2"/>
     </row>
     <row r="23" spans="1:10" ht="6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1434,7 +1437,7 @@
     <row r="24" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="83"/>
-      <c r="C24" s="53" t="s">
+      <c r="C24" s="52" t="s">
         <v>26</v>
       </c>
       <c r="D24" s="7">
@@ -1453,12 +1456,12 @@
     <row r="25" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="84"/>
-      <c r="C25" s="31" t="s">
+      <c r="C25" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="D25" s="27"/>
-      <c r="E25" s="27"/>
-      <c r="F25" s="27"/>
+      <c r="D25" s="26"/>
+      <c r="E25" s="26"/>
+      <c r="F25" s="26"/>
       <c r="G25" s="2"/>
     </row>
     <row r="26" spans="1:10" ht="6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1474,8 +1477,8 @@
     <row r="27" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="83"/>
-      <c r="C27" s="53" t="s">
-        <v>32</v>
+      <c r="C27" s="52" t="s">
+        <v>30</v>
       </c>
       <c r="D27" s="7">
         <v>20</v>
@@ -1493,14 +1496,14 @@
     <row r="28" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="84"/>
-      <c r="C28" s="31" t="s">
-        <v>47</v>
-      </c>
-      <c r="D28" s="27"/>
-      <c r="E28" s="27"/>
-      <c r="F28" s="27"/>
+      <c r="C28" s="30" t="s">
+        <v>45</v>
+      </c>
+      <c r="D28" s="26"/>
+      <c r="E28" s="26"/>
+      <c r="F28" s="26"/>
       <c r="G28" s="2"/>
-      <c r="J28" s="74"/>
+      <c r="J28" s="73"/>
     </row>
     <row r="29" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
@@ -1615,18 +1618,18 @@
       <c r="G56" s="2"/>
     </row>
     <row r="57" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A57" s="39"/>
-      <c r="B57" s="40"/>
-      <c r="C57" s="40"/>
-      <c r="D57" s="41" t="s">
-        <v>49</v>
-      </c>
-      <c r="E57" s="41"/>
-      <c r="F57" s="42">
+      <c r="A57" s="38"/>
+      <c r="B57" s="39"/>
+      <c r="C57" s="39"/>
+      <c r="D57" s="40" t="s">
+        <v>47</v>
+      </c>
+      <c r="E57" s="40"/>
+      <c r="F57" s="41">
         <f>SUM(F15,F18,F21,F6,F24,F27)</f>
         <v>870.30492000000004</v>
       </c>
-      <c r="G57" s="43"/>
+      <c r="G57" s="42"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58" s="1"/>
@@ -1634,7 +1637,7 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" s="76" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B59" s="77"/>
       <c r="C59" s="77"/>
@@ -1644,26 +1647,26 @@
       <c r="G59" s="78"/>
     </row>
     <row r="60" spans="1:7" ht="5.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="28"/>
-      <c r="B60" s="29"/>
-      <c r="C60" s="29"/>
-      <c r="D60" s="29"/>
-      <c r="E60" s="29"/>
-      <c r="F60" s="29"/>
-      <c r="G60" s="30"/>
+      <c r="A60" s="27"/>
+      <c r="B60" s="28"/>
+      <c r="C60" s="28"/>
+      <c r="D60" s="28"/>
+      <c r="E60" s="28"/>
+      <c r="F60" s="28"/>
+      <c r="G60" s="29"/>
     </row>
     <row r="61" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A61" s="44"/>
-      <c r="B61" s="45" t="s">
+      <c r="A61" s="43"/>
+      <c r="B61" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="C61" s="46"/>
+      <c r="C61" s="45"/>
       <c r="D61" s="79" t="s">
         <v>7</v>
       </c>
       <c r="E61" s="79"/>
       <c r="F61" s="79"/>
-      <c r="G61" s="47"/>
+      <c r="G61" s="46"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -1698,60 +1701,60 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7" ht="18" x14ac:dyDescent="0.35">
-      <c r="B2" s="59" t="s">
+      <c r="B2" s="58" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B4" s="59" t="s">
+        <v>32</v>
+      </c>
+      <c r="C4" s="60">
+        <v>0.23</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B6" s="62" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="4" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B4" s="60" t="s">
+      <c r="C6" s="61" t="s">
         <v>34</v>
       </c>
-      <c r="C4" s="61">
-        <v>0.23</v>
-      </c>
-    </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B6" s="63" t="s">
+      <c r="D6" s="62" t="s">
         <v>35</v>
       </c>
-      <c r="C6" s="62" t="s">
+      <c r="E6" s="62" t="s">
         <v>36</v>
       </c>
-      <c r="D6" s="63" t="s">
+      <c r="F6" s="62" t="s">
         <v>37</v>
       </c>
-      <c r="E6" s="63" t="s">
+      <c r="G6" s="62" t="s">
         <v>38</v>
       </c>
-      <c r="F6" s="63" t="s">
-        <v>39</v>
-      </c>
-      <c r="G6" s="63" t="s">
-        <v>40</v>
-      </c>
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B7" s="64">
+      <c r="B7" s="63">
         <f>'PROJETO DE AUDIO'!B11</f>
         <v>1</v>
       </c>
       <c r="C7" t="str">
         <f>'PROJETO DE AUDIO'!C12&amp;" "&amp;'PROJETO DE AUDIO'!C13</f>
-        <v>Behringer Xenyx  X1832USB</v>
-      </c>
-      <c r="D7" s="65"/>
-      <c r="E7" s="65"/>
-      <c r="F7" s="65">
+        <v xml:space="preserve">Behringer Xenyx X2442 USB Aconselhada pelo projetista, mais saidas e maior compatibilidade </v>
+      </c>
+      <c r="D7" s="64"/>
+      <c r="E7" s="64"/>
+      <c r="F7" s="64">
         <f t="shared" ref="F7:F13" si="0">E7*$C$4</f>
         <v>0</v>
       </c>
-      <c r="G7" s="65">
+      <c r="G7" s="64">
         <f t="shared" ref="G7:G13" si="1">E7+F7</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B8" s="64">
+      <c r="B8" s="63">
         <f>'PROJETO DE AUDIO'!B14</f>
         <v>2</v>
       </c>
@@ -1759,25 +1762,25 @@
         <f>'PROJETO DE AUDIO'!C15&amp;" "&amp;'PROJETO DE AUDIO'!C16</f>
         <v>Audibax Arkansas 8 Coluna ativa 2 vias 8" c/ Bluetooth, 80W RMS, XLR/RCA/1/8"</v>
       </c>
-      <c r="D8" s="65">
+      <c r="D8" s="64">
         <f>'PROJETO DE AUDIO'!D15</f>
         <v>101</v>
       </c>
-      <c r="E8" s="65">
+      <c r="E8" s="64">
         <f>'PROJETO DE AUDIO'!E15</f>
         <v>202</v>
       </c>
-      <c r="F8" s="65">
+      <c r="F8" s="64">
         <f t="shared" si="0"/>
         <v>46.46</v>
       </c>
-      <c r="G8" s="65">
+      <c r="G8" s="64">
         <f t="shared" si="1"/>
         <v>248.46</v>
       </c>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B9" s="64">
+      <c r="B9" s="63">
         <f>'PROJETO DE AUDIO'!B17</f>
         <v>1</v>
       </c>
@@ -1785,25 +1788,25 @@
         <f>'PROJETO DE AUDIO'!C18&amp;" "&amp;'PROJETO DE AUDIO'!C19</f>
         <v>Audibax MC XLR 164 30 Stage Box 30m — 16 ins / 4 outs</v>
       </c>
-      <c r="D9" s="65">
+      <c r="D9" s="64">
         <f>'PROJETO DE AUDIO'!D18</f>
         <v>158.00399999999999</v>
       </c>
-      <c r="E9" s="65">
+      <c r="E9" s="64">
         <f>'PROJETO DE AUDIO'!E18</f>
         <v>158.00399999999999</v>
       </c>
-      <c r="F9" s="65">
+      <c r="F9" s="64">
         <f t="shared" si="0"/>
         <v>36.340919999999997</v>
       </c>
-      <c r="G9" s="65">
+      <c r="G9" s="64">
         <f t="shared" si="1"/>
         <v>194.34492</v>
       </c>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B10" s="64">
+      <c r="B10" s="63">
         <f>'PROJETO DE AUDIO'!B20</f>
         <v>4</v>
       </c>
@@ -1811,25 +1814,25 @@
         <f>'PROJETO DE AUDIO'!C21&amp;" "&amp;'PROJETO DE AUDIO'!C22</f>
         <v>Cabo XLR/XLR 50m 3-Pin XLR c/ fichas Amphenol</v>
       </c>
-      <c r="D10" s="65">
+      <c r="D10" s="64">
         <f>'PROJETO DE AUDIO'!D21</f>
         <v>62.498736990179999</v>
       </c>
-      <c r="E10" s="65">
+      <c r="E10" s="64">
         <f>'PROJETO DE AUDIO'!E21</f>
         <v>250</v>
       </c>
-      <c r="F10" s="65">
+      <c r="F10" s="64">
         <f t="shared" si="0"/>
         <v>57.5</v>
       </c>
-      <c r="G10" s="65">
+      <c r="G10" s="64">
         <f t="shared" si="1"/>
         <v>307.5</v>
       </c>
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B11" s="64">
+      <c r="B11" s="63">
         <f>'PROJETO DE AUDIO'!B23</f>
         <v>1</v>
       </c>
@@ -1837,25 +1840,25 @@
         <f>'PROJETO DE AUDIO'!C24&amp;" "&amp;'PROJETO DE AUDIO'!C25</f>
         <v>Restauro e Reabilitação de Coluna Parte elétrica e estrutural</v>
       </c>
-      <c r="D11" s="65">
+      <c r="D11" s="64">
         <f>'PROJETO DE AUDIO'!D24</f>
         <v>90</v>
       </c>
-      <c r="E11" s="65">
+      <c r="E11" s="64">
         <f>'PROJETO DE AUDIO'!E24</f>
         <v>90</v>
       </c>
-      <c r="F11" s="65">
+      <c r="F11" s="64">
         <f t="shared" si="0"/>
         <v>20.7</v>
       </c>
-      <c r="G11" s="65">
+      <c r="G11" s="64">
         <f t="shared" si="1"/>
         <v>110.7</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B12" s="64">
+      <c r="B12" s="63">
         <f>'PROJETO DE AUDIO'!B26</f>
         <v>1</v>
       </c>
@@ -1863,81 +1866,81 @@
         <f>'PROJETO DE AUDIO'!C27&amp;" "&amp;'PROJETO DE AUDIO'!C28</f>
         <v>Acessórios de montagem Abraçadeiras de aluminio/plástico, Fita Termo Retratil, etc.</v>
       </c>
-      <c r="D12" s="65">
+      <c r="D12" s="64">
         <f>'PROJETO DE AUDIO'!D27</f>
         <v>20</v>
       </c>
-      <c r="E12" s="65">
+      <c r="E12" s="64">
         <f>'PROJETO DE AUDIO'!E27</f>
         <v>20</v>
       </c>
-      <c r="F12" s="65">
+      <c r="F12" s="64">
         <f t="shared" si="0"/>
         <v>4.6000000000000005</v>
       </c>
-      <c r="G12" s="65">
+      <c r="G12" s="64">
         <f t="shared" si="1"/>
         <v>24.6</v>
       </c>
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="C13" s="66" t="s">
-        <v>41</v>
-      </c>
-      <c r="E13" s="65">
+      <c r="C13" s="65" t="s">
+        <v>39</v>
+      </c>
+      <c r="E13" s="64">
         <f>'PROJETO DE AUDIO'!F6</f>
         <v>10</v>
       </c>
-      <c r="F13" s="65">
+      <c r="F13" s="64">
         <f t="shared" si="0"/>
         <v>2.3000000000000003</v>
       </c>
-      <c r="G13" s="65">
+      <c r="G13" s="64">
         <f t="shared" si="1"/>
         <v>12.3</v>
       </c>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="C15" s="67" t="s">
-        <v>42</v>
-      </c>
-      <c r="D15" s="68"/>
-      <c r="E15" s="69">
+      <c r="C15" s="66" t="s">
+        <v>40</v>
+      </c>
+      <c r="D15" s="67"/>
+      <c r="E15" s="68">
         <f>SUM(E7:E13)</f>
         <v>730.00400000000002</v>
       </c>
-      <c r="F15" s="69">
+      <c r="F15" s="68">
         <f>SUM(F7:F13)</f>
         <v>167.90091999999999</v>
       </c>
-      <c r="G15" s="70">
+      <c r="G15" s="69">
         <f>SUM(G7:G13)</f>
         <v>897.90492000000006</v>
       </c>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B17" s="60" t="s">
-        <v>43</v>
-      </c>
-      <c r="C17" s="71">
+      <c r="B17" s="59" t="s">
+        <v>41</v>
+      </c>
+      <c r="C17" s="70">
         <f>E15</f>
         <v>730.00400000000002</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B18" s="60" t="s">
-        <v>44</v>
-      </c>
-      <c r="C18" s="71">
+      <c r="B18" s="59" t="s">
+        <v>42</v>
+      </c>
+      <c r="C18" s="70">
         <f>F15</f>
         <v>167.90091999999999</v>
       </c>
     </row>
     <row r="19" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B19" s="72" t="s">
-        <v>45</v>
-      </c>
-      <c r="C19" s="73">
+      <c r="B19" s="71" t="s">
+        <v>43</v>
+      </c>
+      <c r="C19" s="72">
         <f>G15</f>
         <v>897.90492000000006</v>
       </c>

</xml_diff>